<commit_message>
Update PLL_A45 to Fvco 3000 MHz for 600/500 MHz outputs
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013AFX1ASxrYnaovnTssi16w
</commit_message>
<xml_diff>
--- a/pll_cfg.xlsx
+++ b/pll_cfg.xlsx
@@ -598,7 +598,7 @@
         <v>24</v>
       </c>
       <c r="C4" s="4" t="n">
-        <v>100</v>
+        <v>125</v>
       </c>
       <c r="D4" s="4" t="n">
         <v>0</v>
@@ -611,7 +611,7 @@
         <v/>
       </c>
       <c r="G4" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H4" s="3" t="n">
         <v>0</v>
@@ -652,7 +652,7 @@
         <v/>
       </c>
       <c r="J5" s="3" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="K5" s="3" t="n"/>
       <c r="L5" s="3" t="n"/>

</xml_diff>